<commit_message>
docs(backlog): regenerate CAA 311026 with the three proposed estimates
Exported from the backlog Markdown with scripts/export_backlog_xlsx.py --date 311026. Compared with main's workbook, exactly 12 cells change (Points and User Story for E03-S09, E07-S08 and E08-S06 on both sheets); styles, widths and dimensions unchanged. source-of-truth.md already points at CAA 311026.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CONNECTSPHERE BACKLOGS CAA 311026.xlsx
+++ b/docs/CONNECTSPHERE BACKLOGS CAA 311026.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="RELEASE 1 BACKLOG" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="PRODUCT BACKLOG" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RELEASE 1 BACKLOG" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PRODUCT BACKLOG" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1628,7 +1628,8 @@
       <c r="E22" s="2" t="inlineStr">
         <is>
           <t>As an Event Coordinator Lead, I want to reassign an event to a different Event Coordinator where necessary so that workload, absences and conflicts can be managed without waiting on the current Coordinator.
-New story from the Week 7 Customer Changes (C-69). The Coordinator-initiated reassignment with acceptance delivered by E03-S01 Scenarios 3 to 6 stays in force (T-15 amended, not replaced). Estimate at Sprint 3 planning (T-73). Scenarios tagged "(assumes O-xx)" are written to the default recorded in `docs/bdr/C-open-questions.md`.</t>
+New story from the Week 7 Customer Changes (C-69). The Coordinator-initiated reassignment with acceptance delivered by E03-S01 Scenarios 3 to 6 stays in force (T-15 amended, not replaced). Estimate at Sprint 3 planning (T-73). Scenarios tagged "(assumes O-xx)" are written to the default recorded in `docs/bdr/C-open-questions.md`.
+No estimate was recorded at Sprint 3 planning. A three-point estimate was proposed on 31 October 2026 for teammate/PO review, sized against E03-S01 Coordinator assignment (3) and E03-S02 clarification requests (3): the Lead's immediate reassignment with notices to both Coordinators and the Organiser and an activity-log entry, a new request-to-the-Lead path with decline, and a role refusal. Scenario 2 reuses E03-S01 unchanged and is not counted again. Jira stays blank until this backlog PR merges and the estimate is accepted. T-73 estimates in-flight stories for their remaining work only; this story is not yet in flight, so the size is a whole-story reference, and team/PO confirmation is required on how it is counted for sprint reporting. This proposal does not change the sprint, owner, accepted criteria or history.</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
@@ -1648,7 +1649,9 @@
 - Be refused when attempting to reassign an event I am not assigned to and am not the Lead for</t>
         </is>
       </c>
-      <c r="G22" s="2" t="inlineStr"/>
+      <c r="G22" s="2" t="n">
+        <v>3</v>
+      </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
           <t>C-69, C-56, T-15, T-70, T-73, T-74, O-36, O-37</t>
@@ -3016,7 +3019,8 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>As a Technical Support Staff member, I want equipment requests and reservations to identify the Session they support so that availability and fulfilment use the correct Session period.</t>
+          <t>As a Technical Support Staff member, I want equipment requests and reservations to identify the Session they support so that availability and fulfilment use the correct Session period.
+No estimate was previously recorded. A three-point estimate was proposed on 31 October 2026 for teammate/PO review, sized against E07-S02 equipment requests (3), E07-S04 equipment reservations (5) and E02-S07 date horizon (3): a Session link on equipment requests and reservations, availability checked on the Session period, cross-event refusal, and event-level staff assignment left unchanged. The E04-S02 Session write path is a dependency, not work counted again here. Jira stays blank until this backlog PR merges and the estimate is accepted. T-73 estimates in-flight stories for their remaining work only; this story is not yet in flight, so the size is a whole-story reference, and team/PO confirmation is required on how it is counted for sprint reporting. This proposal does not change the sprint, owner, accepted criteria or history.</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
@@ -3036,7 +3040,9 @@
 - Keep technical-support staff assignment event-level</t>
         </is>
       </c>
-      <c r="G46" s="2" t="inlineStr"/>
+      <c r="G46" s="2" t="n">
+        <v>3</v>
+      </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
           <t>C-107, T-74, T-79</t>
@@ -3288,7 +3294,8 @@
       <c r="E51" s="2" t="inlineStr">
         <is>
           <t>As a Safety Officer, I want to review the operational safety of each event whose venue and technical arrangements are confirmed, and approve it, reject its safety arrangement or request changes, so that no event proceeds to preparation until it is safe to run.
-New story from the Week 7 Customer Changes (C-70) and the seventh role (T-72). The Safety Review status it works on sits between Planning and Confirmed as an interim placement (T-71); O-39 asks the customer to confirm. The customer guarantees a response, so there is no timeout path. Estimate at Sprint 3 planning (T-73). Scenarios tagged "(assumes O-xx)" are written to the default recorded in `docs/bdr/C-open-questions.md`.</t>
+New story from the Week 7 Customer Changes (C-70) and the seventh role (T-72). The Safety Review status it works on sits between Planning and Confirmed as an interim placement (T-71); O-39 asks the customer to confirm. The customer guarantees a response, so there is no timeout path. Estimate at Sprint 3 planning (T-73). Scenarios tagged "(assumes O-xx)" are written to the default recorded in `docs/bdr/C-open-questions.md`.
+No estimate was recorded at Sprint 3 planning. An eight-point estimate was proposed on 31 October 2026 for teammate/PO review, sized against E08-S03 event confirmation (5), E10-S01 change requests (8) and E05-S06 venue unavailability (8): ten scenarios across backend and frontend, covering a new Safety Officer queue, a seven-factor checklist, approve, request-changes and reject decisions with status changes, re-review flags, notices, audit entries and status-display and deactivation changes. The Safety Review status, migration 0017 and the submission step already delivered by other stories (#282, #283) are not counted. Jira stays blank until this backlog PR merges and the estimate is accepted. T-73 estimates in-flight stories for their remaining work only; this story is not yet in flight, so the size is a whole-story reference, and team/PO confirmation is required on how it is counted for sprint reporting. This proposal does not change the sprint, owner, accepted criteria or history.</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
@@ -3324,7 +3331,9 @@
 - Confirm every decision is in the activity log</t>
         </is>
       </c>
-      <c r="G51" s="2" t="inlineStr"/>
+      <c r="G51" s="2" t="n">
+        <v>8</v>
+      </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
           <t>C-70, T-71, T-72, T-73, T-74, O-39, O-40, O-41, O-42, O-43</t>
@@ -5486,7 +5495,8 @@
       <c r="E28" s="2" t="inlineStr">
         <is>
           <t>As an Event Coordinator Lead, I want to reassign an event to a different Event Coordinator where necessary so that workload, absences and conflicts can be managed without waiting on the current Coordinator.
-New story from the Week 7 Customer Changes (C-69). The Coordinator-initiated reassignment with acceptance delivered by E03-S01 Scenarios 3 to 6 stays in force (T-15 amended, not replaced). Estimate at Sprint 3 planning (T-73). Scenarios tagged "(assumes O-xx)" are written to the default recorded in `docs/bdr/C-open-questions.md`.</t>
+New story from the Week 7 Customer Changes (C-69). The Coordinator-initiated reassignment with acceptance delivered by E03-S01 Scenarios 3 to 6 stays in force (T-15 amended, not replaced). Estimate at Sprint 3 planning (T-73). Scenarios tagged "(assumes O-xx)" are written to the default recorded in `docs/bdr/C-open-questions.md`.
+No estimate was recorded at Sprint 3 planning. A three-point estimate was proposed on 31 October 2026 for teammate/PO review, sized against E03-S01 Coordinator assignment (3) and E03-S02 clarification requests (3): the Lead's immediate reassignment with notices to both Coordinators and the Organiser and an activity-log entry, a new request-to-the-Lead path with decline, and a role refusal. Scenario 2 reuses E03-S01 unchanged and is not counted again. Jira stays blank until this backlog PR merges and the estimate is accepted. T-73 estimates in-flight stories for their remaining work only; this story is not yet in flight, so the size is a whole-story reference, and team/PO confirmation is required on how it is counted for sprint reporting. This proposal does not change the sprint, owner, accepted criteria or history.</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
@@ -5506,7 +5516,9 @@
 - Be refused when attempting to reassign an event I am not assigned to and am not the Lead for</t>
         </is>
       </c>
-      <c r="G28" s="2" t="inlineStr"/>
+      <c r="G28" s="2" t="n">
+        <v>3</v>
+      </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
           <t>C-69, C-56, T-15, T-70, T-73, T-74, O-36, O-37</t>
@@ -6808,7 +6820,8 @@
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>As a Technical Support Staff member, I want equipment requests and reservations to identify the Session they support so that availability and fulfilment use the correct Session period.</t>
+          <t>As a Technical Support Staff member, I want equipment requests and reservations to identify the Session they support so that availability and fulfilment use the correct Session period.
+No estimate was previously recorded. A three-point estimate was proposed on 31 October 2026 for teammate/PO review, sized against E07-S02 equipment requests (3), E07-S04 equipment reservations (5) and E02-S07 date horizon (3): a Session link on equipment requests and reservations, availability checked on the Session period, cross-event refusal, and event-level staff assignment left unchanged. The E04-S02 Session write path is a dependency, not work counted again here. Jira stays blank until this backlog PR merges and the estimate is accepted. T-73 estimates in-flight stories for their remaining work only; this story is not yet in flight, so the size is a whole-story reference, and team/PO confirmation is required on how it is counted for sprint reporting. This proposal does not change the sprint, owner, accepted criteria or history.</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
@@ -6828,7 +6841,9 @@
 - Keep technical-support staff assignment event-level</t>
         </is>
       </c>
-      <c r="G53" s="2" t="inlineStr"/>
+      <c r="G53" s="2" t="n">
+        <v>3</v>
+      </c>
       <c r="H53" s="2" t="inlineStr">
         <is>
           <t>C-107, T-74, T-79</t>
@@ -7144,7 +7159,8 @@
       <c r="E60" s="2" t="inlineStr">
         <is>
           <t>As a Safety Officer, I want to review the operational safety of each event whose venue and technical arrangements are confirmed, and approve it, reject its safety arrangement or request changes, so that no event proceeds to preparation until it is safe to run.
-New story from the Week 7 Customer Changes (C-70) and the seventh role (T-72). The Safety Review status it works on sits between Planning and Confirmed as an interim placement (T-71); O-39 asks the customer to confirm. The customer guarantees a response, so there is no timeout path. Estimate at Sprint 3 planning (T-73). Scenarios tagged "(assumes O-xx)" are written to the default recorded in `docs/bdr/C-open-questions.md`.</t>
+New story from the Week 7 Customer Changes (C-70) and the seventh role (T-72). The Safety Review status it works on sits between Planning and Confirmed as an interim placement (T-71); O-39 asks the customer to confirm. The customer guarantees a response, so there is no timeout path. Estimate at Sprint 3 planning (T-73). Scenarios tagged "(assumes O-xx)" are written to the default recorded in `docs/bdr/C-open-questions.md`.
+No estimate was recorded at Sprint 3 planning. An eight-point estimate was proposed on 31 October 2026 for teammate/PO review, sized against E08-S03 event confirmation (5), E10-S01 change requests (8) and E05-S06 venue unavailability (8): ten scenarios across backend and frontend, covering a new Safety Officer queue, a seven-factor checklist, approve, request-changes and reject decisions with status changes, re-review flags, notices, audit entries and status-display and deactivation changes. The Safety Review status, migration 0017 and the submission step already delivered by other stories (#282, #283) are not counted. Jira stays blank until this backlog PR merges and the estimate is accepted. T-73 estimates in-flight stories for their remaining work only; this story is not yet in flight, so the size is a whole-story reference, and team/PO confirmation is required on how it is counted for sprint reporting. This proposal does not change the sprint, owner, accepted criteria or history.</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
@@ -7180,7 +7196,9 @@
 - Confirm every decision is in the activity log</t>
         </is>
       </c>
-      <c r="G60" s="2" t="inlineStr"/>
+      <c r="G60" s="2" t="n">
+        <v>8</v>
+      </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
           <t>C-70, T-71, T-72, T-73, T-74, O-39, O-40, O-41, O-42, O-43</t>

</xml_diff>

<commit_message>
docs(backlog): flag Technical Support staffing on date changes in E10-S02 (SCRUM-244)
PO answer on 31 October (T-103), after the E08-S04 manual run showed a moved
event entering Safety Review with its support crew still on the old day.
E10-S02 is In Progress, so Scenarios 5 and 6 and the checklist are updated
in place in both backlog views (T-74) and the story is re-estimated from 5
to 8 points by its owner (T-37, T-73). Backlog workbook re-exported; handoff
started for SCRUM-244.
</commit_message>
<xml_diff>
--- a/docs/CONNECTSPHERE BACKLOGS CAA 311026.xlsx
+++ b/docs/CONNECTSPHERE BACKLOGS CAA 311026.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="RELEASE 1 BACKLOG" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="PRODUCT BACKLOG" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RELEASE 1 BACKLOG" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PRODUCT BACKLOG" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3810,24 +3810,25 @@
 Scenario 4 - Over-subscription warns only
 Given a change would make a Session or combined Event registration capacity lower than approved registrations When the change is saved Then I am warned and shown the over-subscription, and no Attendee is automatically removed or waitlisted
 Scenario 5 - Session date/time change flags its arrangements
-Given a Session date or time changes When the change takes effect Then that Session's venue booking and equipment reservations are flagged for reconfirmation; an Event-wide date/time change flags all of its Session arrangements
+Given a Session date or time changes When the change takes effect Then that Session's venue booking and equipment reservations, and any staffed Technical Support request overlapping its previous time, are flagged for reconfirmation; an Event-wide date/time change flags all of its Session arrangements and every staffed Technical Support request; a flagged Technical Support request counts as outstanding for readiness until Technical Support Staff reconfirm it at the new time (T-103)
 Scenario 6 - Affected staff notified
-Given a change flags a venue or equipment arrangement When the affected arrangements are identified Then the assigned Venue Staff and Technical Support Staff are notified
+Given a change flags a venue, equipment or Technical Support staffing arrangement When the affected arrangements are identified Then the assigned Venue Staff and Technical Support Staff are notified
 Checklist
 - Flag only the Session arrangement whose governing headcount exceeds capacity
 - Leave arrangements unflagged for description-only edits
 - Show affected Session bookings/reservations before applying a change
 - Warn about over-subscription without automatically removing or waitlisting Attendees
 - Flag the affected Session or all Sessions for date/time changes as appropriate
+- Flag staffed Technical Support requests on a date/time change and let Technical Support Staff reconfirm them at the new time (T-103)
 - Notify staff responsible for the affected arrangements</t>
         </is>
       </c>
       <c r="G60" s="2" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
-          <t>C-05, T-16, B-05, B-11, C-67, T-68, O-27, C-107, T-79</t>
+          <t>C-05, T-16, B-05, B-11, C-67, T-68, O-27, C-107, T-79, T-103</t>
         </is>
       </c>
       <c r="I60" s="2" t="inlineStr"/>
@@ -7630,24 +7631,25 @@
 Scenario 4 - Over-subscription warns only
 Given a change would make a Session or combined Event registration capacity lower than approved registrations When the change is saved Then I am warned and shown the over-subscription, and no Attendee is automatically removed or waitlisted
 Scenario 5 - Session date/time change flags its arrangements
-Given a Session date or time changes When the change takes effect Then that Session's venue booking and equipment reservations are flagged for reconfirmation; an Event-wide date/time change flags all of its Session arrangements
+Given a Session date or time changes When the change takes effect Then that Session's venue booking and equipment reservations, and any staffed Technical Support request overlapping its previous time, are flagged for reconfirmation; an Event-wide date/time change flags all of its Session arrangements and every staffed Technical Support request; a flagged Technical Support request counts as outstanding for readiness until Technical Support Staff reconfirm it at the new time (T-103)
 Scenario 6 - Affected staff notified
-Given a change flags a venue or equipment arrangement When the affected arrangements are identified Then the assigned Venue Staff and Technical Support Staff are notified
+Given a change flags a venue, equipment or Technical Support staffing arrangement When the affected arrangements are identified Then the assigned Venue Staff and Technical Support Staff are notified
 Checklist
 - Flag only the Session arrangement whose governing headcount exceeds capacity
 - Leave arrangements unflagged for description-only edits
 - Show affected Session bookings/reservations before applying a change
 - Warn about over-subscription without automatically removing or waitlisting Attendees
 - Flag the affected Session or all Sessions for date/time changes as appropriate
+- Flag staffed Technical Support requests on a date/time change and let Technical Support Staff reconfirm them at the new time (T-103)
 - Notify staff responsible for the affected arrangements</t>
         </is>
       </c>
       <c r="G69" s="2" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="H69" s="2" t="inlineStr">
         <is>
-          <t>C-05, T-16, B-05, B-11, C-67, T-68, O-27, C-107, T-79</t>
+          <t>C-05, T-16, B-05, B-11, C-67, T-68, O-27, C-107, T-79, T-103</t>
         </is>
       </c>
       <c r="I69" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
docs(backlog): align E10-S02 Scenario 3 and its cases with T-103 (SCRUM-244)
T-103 says a flagged Technical Support request is listed in the change
preview; Scenario 3 now names it in both backlog views and the workbook,
and TC_E10S02_03 says the same. TC_E10S02_01 loses a leftover second
block that filled its exported steps and result with an older
single-Session case; TC_E10S02_05's AC reference adds T-103.
</commit_message>
<xml_diff>
--- a/docs/CONNECTSPHERE BACKLOGS CAA 311026.xlsx
+++ b/docs/CONNECTSPHERE BACKLOGS CAA 311026.xlsx
@@ -3806,7 +3806,7 @@
 Scenario 2 - Description-only edit flags nothing
 Given an Event has confirmed venue and equipment arrangements When only its Event description is edited Then no arrangements are flagged
 Scenario 3 - Affected Session arrangements shown first
-Given a change affects confirmed arrangements When I save it Then I am shown the affected Session bookings and equipment reservations before the change takes effect
+Given a change affects confirmed arrangements When I save it Then I am shown the affected Session bookings, equipment reservations and staffed Technical Support requests before the change takes effect (T-103)
 Scenario 4 - Over-subscription warns only
 Given a change would make a Session or combined Event registration capacity lower than approved registrations When the change is saved Then I am warned and shown the over-subscription, and no Attendee is automatically removed or waitlisted
 Scenario 5 - Session date/time change flags its arrangements
@@ -7627,7 +7627,7 @@
 Scenario 2 - Description-only edit flags nothing
 Given an Event has confirmed venue and equipment arrangements When only its Event description is edited Then no arrangements are flagged
 Scenario 3 - Affected Session arrangements shown first
-Given a change affects confirmed arrangements When I save it Then I am shown the affected Session bookings and equipment reservations before the change takes effect
+Given a change affects confirmed arrangements When I save it Then I am shown the affected Session bookings, equipment reservations and staffed Technical Support requests before the change takes effect (T-103)
 Scenario 4 - Over-subscription warns only
 Given a change would make a Session or combined Event registration capacity lower than approved registrations When the change is saved Then I am warned and shown the over-subscription, and no Attendee is automatically removed or waitlisted
 Scenario 5 - Session date/time change flags its arrangements

</xml_diff>

<commit_message>
docs(backlog): add T-103 Technical Support reconfirmation to E10-S02 (SCRUM-244)
The Product Owner answered yes on 31 October (question on #392): a date
or time change also flags staffed Technical Support for reconfirmation.
E10-S02 Scenarios 3, 5 and 6 and the checklist are updated in place in
both backlog views, the story is re-estimated from 5 to 8 points, and its
test cases cover the new criteria (TC_E10S02_10 to _13 added; _03, _05,
_06 and _08 extended). Workbooks and tc-coverage regenerated.
</commit_message>
<xml_diff>
--- a/docs/CONNECTSPHERE BACKLOGS CAA 311026.xlsx
+++ b/docs/CONNECTSPHERE BACKLOGS CAA 311026.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="RELEASE 1 BACKLOG" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="PRODUCT BACKLOG" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RELEASE 1 BACKLOG" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PRODUCT BACKLOG" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3806,28 +3806,29 @@
 Scenario 2 - Description-only edit flags nothing
 Given an Event has confirmed venue and equipment arrangements When only its Event description is edited Then no arrangements are flagged
 Scenario 3 - Affected Session arrangements shown first
-Given a change affects confirmed arrangements When I save it Then I am shown the affected Session bookings and equipment reservations before the change takes effect
+Given a change affects confirmed arrangements When I save it Then I am shown the affected Session bookings, equipment reservations and staffed Technical Support requests before the change takes effect (T-103)
 Scenario 4 - Over-subscription warns only
 Given a change would make a Session or combined Event registration capacity lower than approved registrations When the change is saved Then I am warned and shown the over-subscription, and no Attendee is automatically removed or waitlisted
 Scenario 5 - Session date/time change flags its arrangements
-Given a Session date or time changes When the change takes effect Then that Session's venue booking and equipment reservations are flagged for reconfirmation; an Event-wide date/time change flags all of its Session arrangements
+Given a Session date or time changes When the change takes effect Then that Session's venue booking and equipment reservations, and any staffed Technical Support request overlapping its previous time, are flagged for reconfirmation; an Event-wide date/time change flags all of its Session arrangements and every staffed Technical Support request; a flagged Technical Support request counts as outstanding for readiness until Technical Support Staff reconfirm it at the new time (T-103)
 Scenario 6 - Affected staff notified
-Given a change flags a venue or equipment arrangement When the affected arrangements are identified Then the assigned Venue Staff and Technical Support Staff are notified
+Given a change flags a venue, equipment or Technical Support staffing arrangement When the affected arrangements are identified Then the assigned Venue Staff and Technical Support Staff are notified
 Checklist
 - Flag only the Session arrangement whose governing headcount exceeds capacity
 - Leave arrangements unflagged for description-only edits
 - Show affected Session bookings/reservations before applying a change
 - Warn about over-subscription without automatically removing or waitlisting Attendees
 - Flag the affected Session or all Sessions for date/time changes as appropriate
+- Flag staffed Technical Support requests on a date/time change and let Technical Support Staff reconfirm them at the new time (T-103)
 - Notify staff responsible for the affected arrangements</t>
         </is>
       </c>
       <c r="G60" s="2" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
-          <t>C-05, T-16, B-05, B-11, C-67, T-68, O-27, C-107, T-79</t>
+          <t>C-05, T-16, B-05, B-11, C-67, T-68, O-27, C-107, T-79, T-103</t>
         </is>
       </c>
       <c r="I60" s="2" t="inlineStr"/>
@@ -7626,28 +7627,29 @@
 Scenario 2 - Description-only edit flags nothing
 Given an Event has confirmed venue and equipment arrangements When only its Event description is edited Then no arrangements are flagged
 Scenario 3 - Affected Session arrangements shown first
-Given a change affects confirmed arrangements When I save it Then I am shown the affected Session bookings and equipment reservations before the change takes effect
+Given a change affects confirmed arrangements When I save it Then I am shown the affected Session bookings, equipment reservations and staffed Technical Support requests before the change takes effect (T-103)
 Scenario 4 - Over-subscription warns only
 Given a change would make a Session or combined Event registration capacity lower than approved registrations When the change is saved Then I am warned and shown the over-subscription, and no Attendee is automatically removed or waitlisted
 Scenario 5 - Session date/time change flags its arrangements
-Given a Session date or time changes When the change takes effect Then that Session's venue booking and equipment reservations are flagged for reconfirmation; an Event-wide date/time change flags all of its Session arrangements
+Given a Session date or time changes When the change takes effect Then that Session's venue booking and equipment reservations, and any staffed Technical Support request overlapping its previous time, are flagged for reconfirmation; an Event-wide date/time change flags all of its Session arrangements and every staffed Technical Support request; a flagged Technical Support request counts as outstanding for readiness until Technical Support Staff reconfirm it at the new time (T-103)
 Scenario 6 - Affected staff notified
-Given a change flags a venue or equipment arrangement When the affected arrangements are identified Then the assigned Venue Staff and Technical Support Staff are notified
+Given a change flags a venue, equipment or Technical Support staffing arrangement When the affected arrangements are identified Then the assigned Venue Staff and Technical Support Staff are notified
 Checklist
 - Flag only the Session arrangement whose governing headcount exceeds capacity
 - Leave arrangements unflagged for description-only edits
 - Show affected Session bookings/reservations before applying a change
 - Warn about over-subscription without automatically removing or waitlisting Attendees
 - Flag the affected Session or all Sessions for date/time changes as appropriate
+- Flag staffed Technical Support requests on a date/time change and let Technical Support Staff reconfirm them at the new time (T-103)
 - Notify staff responsible for the affected arrangements</t>
         </is>
       </c>
       <c r="G69" s="2" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="H69" s="2" t="inlineStr">
         <is>
-          <t>C-05, T-16, B-05, B-11, C-67, T-68, O-27, C-107, T-79</t>
+          <t>C-05, T-16, B-05, B-11, C-67, T-68, O-27, C-107, T-79, T-103</t>
         </is>
       </c>
       <c r="I69" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
docs(backlog): propose thirteen points for E11 notifications
Estimate proposal for E11-S01; SCRUM-75 remains at five pending explicit team/PO agreement and merge. Preserve T-37 scale and T-73 reporting decisions for review; no story closing clause.
</commit_message>
<xml_diff>
--- a/docs/CONNECTSPHERE BACKLOGS CAA 311026.xlsx
+++ b/docs/CONNECTSPHERE BACKLOGS CAA 311026.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="RELEASE 1 BACKLOG" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="PRODUCT BACKLOG" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RELEASE 1 BACKLOG" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PRODUCT BACKLOG" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3968,7 +3968,26 @@
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>As a user involved in an event, I want to be notified when its status or arrangements change so that I do not have to keep checking the system and nobody continues working from outdated information.</t>
+          <t>As a user involved in an event, I want to be notified when its status or arrangements change so that I do not have to keep checking the system and nobody continues working from outdated information.
+Estimate proposal (31 October 2026, for team/PO review): change the full-story
+size from the original five points to thirteen. Jira remains at five until the
+proposal is approved and merged. The routing matrix spans status/booking,
+equipment/support, effective arrangement changes, cancellation and waiting-list
+notifications; implementation includes recipient filtering, actor exclusion,
+deduplication, public/private content boundaries, transactional inbox/outbox,
+email failure handling, inbox/read state, and cross-workflow integration and
+human delivery evidence. Business implementations owned by booking, equipment,
+registration and change-management stories are excluded; only their E11 hooks
+and notification verification are counted here. Waiting time, PR count and work
+already credited elsewhere are not estimation inputs.
+Thirteen is a proposed whole-story sizing correction, not thirteen points of
+remaining work or extra velocity. T-73 sizes in-flight work by the remaining
+work, so team/PO confirmation of the recording/reporting basis is required;
+original sprint commitments and the five-point historical baseline stay intact.
+T-37 currently maps S=1, M=3, L=5 and XL=8: thirteen requires explicit team/PO
+agreement to a larger size or an alternative estimate. This proposal does not
+silently amend T-37 or claim a new size has already been agreed. Acceptance
+criteria, implementation status and final acceptance requirements are unchanged.</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
@@ -4000,7 +4019,7 @@
         </is>
       </c>
       <c r="G63" s="2" t="n">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="H63" s="2" t="inlineStr">
         <is>
@@ -7825,7 +7844,26 @@
       </c>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t>As a user involved in an event, I want to be notified when its status or arrangements change so that I do not have to keep checking the system and nobody continues working from outdated information.</t>
+          <t>As a user involved in an event, I want to be notified when its status or arrangements change so that I do not have to keep checking the system and nobody continues working from outdated information.
+Estimate proposal (31 October 2026, for team/PO review): change the full-story
+size from the original five points to thirteen. Jira remains at five until the
+proposal is approved and merged. The routing matrix spans status/booking,
+equipment/support, effective arrangement changes, cancellation and waiting-list
+notifications; implementation includes recipient filtering, actor exclusion,
+deduplication, public/private content boundaries, transactional inbox/outbox,
+email failure handling, inbox/read state, and cross-workflow integration and
+human delivery evidence. Business implementations owned by booking, equipment,
+registration and change-management stories are excluded; only their E11 hooks
+and notification verification are counted here. Waiting time, PR count and work
+already credited elsewhere are not estimation inputs.
+Thirteen is a proposed whole-story sizing correction, not thirteen points of
+remaining work or extra velocity. T-73 sizes in-flight work by the remaining
+work, so team/PO confirmation of the recording/reporting basis is required;
+original sprint commitments and the five-point historical baseline stay intact.
+T-37 currently maps S=1, M=3, L=5 and XL=8: thirteen requires explicit team/PO
+agreement to a larger size or an alternative estimate. This proposal does not
+silently amend T-37 or claim a new size has already been agreed. Acceptance
+criteria, implementation status and final acceptance requirements are unchanged.</t>
         </is>
       </c>
       <c r="F73" s="2" t="inlineStr">
@@ -7857,7 +7895,7 @@
         </is>
       </c>
       <c r="G73" s="2" t="n">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="H73" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
docs(bdr): renumber the Technical Support decision to T-104 (SCRUM-244)
Ji Ning's #395 also records a T-103 (affected approved changes interrupt Safety Review) and merges first, so this decision takes the next number. References, workbooks and tc-coverage updated.
</commit_message>
<xml_diff>
--- a/docs/CONNECTSPHERE BACKLOGS CAA 311026.xlsx
+++ b/docs/CONNECTSPHERE BACKLOGS CAA 311026.xlsx
@@ -3806,11 +3806,11 @@
 Scenario 2 - Description-only edit flags nothing
 Given an Event has confirmed venue and equipment arrangements When only its Event description is edited Then no arrangements are flagged
 Scenario 3 - Affected Session arrangements shown first
-Given a change affects confirmed arrangements When I save it Then I am shown the affected Session bookings, equipment reservations and staffed Technical Support requests before the change takes effect (T-103)
+Given a change affects confirmed arrangements When I save it Then I am shown the affected Session bookings, equipment reservations and staffed Technical Support requests before the change takes effect (T-104)
 Scenario 4 - Over-subscription warns only
 Given a change would make a Session or combined Event registration capacity lower than approved registrations When the change is saved Then I am warned and shown the over-subscription, and no Attendee is automatically removed or waitlisted
 Scenario 5 - Session date/time change flags its arrangements
-Given a Session date or time changes When the change takes effect Then that Session's venue booking and equipment reservations, and any staffed Technical Support request overlapping its previous time, are flagged for reconfirmation; an Event-wide date/time change flags all of its Session arrangements and every staffed Technical Support request; a flagged Technical Support request counts as outstanding for readiness until Technical Support Staff reconfirm it at the new time (T-103)
+Given a Session date or time changes When the change takes effect Then that Session's venue booking and equipment reservations, and any staffed Technical Support request overlapping its previous time, are flagged for reconfirmation; an Event-wide date/time change flags all of its Session arrangements and every staffed Technical Support request; a flagged Technical Support request counts as outstanding for readiness until Technical Support Staff reconfirm it at the new time (T-104)
 Scenario 6 - Affected staff notified
 Given a change flags a venue, equipment or Technical Support staffing arrangement When the affected arrangements are identified Then the assigned Venue Staff and Technical Support Staff are notified
 Checklist
@@ -3819,7 +3819,7 @@
 - Show affected Session bookings/reservations before applying a change
 - Warn about over-subscription without automatically removing or waitlisting Attendees
 - Flag the affected Session or all Sessions for date/time changes as appropriate
-- Flag staffed Technical Support requests on a date/time change and let Technical Support Staff reconfirm them at the new time (T-103)
+- Flag staffed Technical Support requests on a date/time change and let Technical Support Staff reconfirm them at the new time (T-104)
 - Notify staff responsible for the affected arrangements</t>
         </is>
       </c>
@@ -3828,7 +3828,7 @@
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
-          <t>C-05, T-16, B-05, B-11, C-67, T-68, O-27, C-107, T-79, T-103</t>
+          <t>C-05, T-16, B-05, B-11, C-67, T-68, O-27, C-107, T-79, T-104</t>
         </is>
       </c>
       <c r="I60" s="2" t="inlineStr"/>
@@ -7627,11 +7627,11 @@
 Scenario 2 - Description-only edit flags nothing
 Given an Event has confirmed venue and equipment arrangements When only its Event description is edited Then no arrangements are flagged
 Scenario 3 - Affected Session arrangements shown first
-Given a change affects confirmed arrangements When I save it Then I am shown the affected Session bookings, equipment reservations and staffed Technical Support requests before the change takes effect (T-103)
+Given a change affects confirmed arrangements When I save it Then I am shown the affected Session bookings, equipment reservations and staffed Technical Support requests before the change takes effect (T-104)
 Scenario 4 - Over-subscription warns only
 Given a change would make a Session or combined Event registration capacity lower than approved registrations When the change is saved Then I am warned and shown the over-subscription, and no Attendee is automatically removed or waitlisted
 Scenario 5 - Session date/time change flags its arrangements
-Given a Session date or time changes When the change takes effect Then that Session's venue booking and equipment reservations, and any staffed Technical Support request overlapping its previous time, are flagged for reconfirmation; an Event-wide date/time change flags all of its Session arrangements and every staffed Technical Support request; a flagged Technical Support request counts as outstanding for readiness until Technical Support Staff reconfirm it at the new time (T-103)
+Given a Session date or time changes When the change takes effect Then that Session's venue booking and equipment reservations, and any staffed Technical Support request overlapping its previous time, are flagged for reconfirmation; an Event-wide date/time change flags all of its Session arrangements and every staffed Technical Support request; a flagged Technical Support request counts as outstanding for readiness until Technical Support Staff reconfirm it at the new time (T-104)
 Scenario 6 - Affected staff notified
 Given a change flags a venue, equipment or Technical Support staffing arrangement When the affected arrangements are identified Then the assigned Venue Staff and Technical Support Staff are notified
 Checklist
@@ -7640,7 +7640,7 @@
 - Show affected Session bookings/reservations before applying a change
 - Warn about over-subscription without automatically removing or waitlisting Attendees
 - Flag the affected Session or all Sessions for date/time changes as appropriate
-- Flag staffed Technical Support requests on a date/time change and let Technical Support Staff reconfirm them at the new time (T-103)
+- Flag staffed Technical Support requests on a date/time change and let Technical Support Staff reconfirm them at the new time (T-104)
 - Notify staff responsible for the affected arrangements</t>
         </is>
       </c>
@@ -7649,7 +7649,7 @@
       </c>
       <c r="H69" s="2" t="inlineStr">
         <is>
-          <t>C-05, T-16, B-05, B-11, C-67, T-68, O-27, C-107, T-79, T-103</t>
+          <t>C-05, T-16, B-05, B-11, C-67, T-68, O-27, C-107, T-79, T-104</t>
         </is>
       </c>
       <c r="I69" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: renumber the Technical Support decision to T-104 (SCRUM-244)
Ji Ning's #395 also records a T-103 (affected approved changes interrupt Safety Review) and merges first. Comments, test titles, docs, workbooks and tc-coverage now say T-104; the committed run records stay as written (T-65).
</commit_message>
<xml_diff>
--- a/docs/CONNECTSPHERE BACKLOGS CAA 311026.xlsx
+++ b/docs/CONNECTSPHERE BACKLOGS CAA 311026.xlsx
@@ -3806,11 +3806,11 @@
 Scenario 2 - Description-only edit flags nothing
 Given an Event has confirmed venue and equipment arrangements When only its Event description is edited Then no arrangements are flagged
 Scenario 3 - Affected Session arrangements shown first
-Given a change affects confirmed arrangements When I save it Then I am shown the affected Session bookings, equipment reservations and staffed Technical Support requests before the change takes effect (T-103)
+Given a change affects confirmed arrangements When I save it Then I am shown the affected Session bookings, equipment reservations and staffed Technical Support requests before the change takes effect (T-104)
 Scenario 4 - Over-subscription warns only
 Given a change would make a Session or combined Event registration capacity lower than approved registrations When the change is saved Then I am warned and shown the over-subscription, and no Attendee is automatically removed or waitlisted
 Scenario 5 - Session date/time change flags its arrangements
-Given a Session date or time changes When the change takes effect Then that Session's venue booking and equipment reservations, and any staffed Technical Support request overlapping its previous time, are flagged for reconfirmation; an Event-wide date/time change flags all of its Session arrangements and every staffed Technical Support request; a flagged Technical Support request counts as outstanding for readiness until Technical Support Staff reconfirm it at the new time (T-103)
+Given a Session date or time changes When the change takes effect Then that Session's venue booking and equipment reservations, and any staffed Technical Support request overlapping its previous time, are flagged for reconfirmation; an Event-wide date/time change flags all of its Session arrangements and every staffed Technical Support request; a flagged Technical Support request counts as outstanding for readiness until Technical Support Staff reconfirm it at the new time (T-104)
 Scenario 6 - Affected staff notified
 Given a change flags a venue, equipment or Technical Support staffing arrangement When the affected arrangements are identified Then the assigned Venue Staff and Technical Support Staff are notified
 Checklist
@@ -3819,7 +3819,7 @@
 - Show affected Session bookings/reservations before applying a change
 - Warn about over-subscription without automatically removing or waitlisting Attendees
 - Flag the affected Session or all Sessions for date/time changes as appropriate
-- Flag staffed Technical Support requests on a date/time change and let Technical Support Staff reconfirm them at the new time (T-103)
+- Flag staffed Technical Support requests on a date/time change and let Technical Support Staff reconfirm them at the new time (T-104)
 - Notify staff responsible for the affected arrangements</t>
         </is>
       </c>
@@ -3828,7 +3828,7 @@
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
-          <t>C-05, T-16, B-05, B-11, C-67, T-68, O-27, C-107, T-79, T-103</t>
+          <t>C-05, T-16, B-05, B-11, C-67, T-68, O-27, C-107, T-79, T-104</t>
         </is>
       </c>
       <c r="I60" s="2" t="inlineStr"/>
@@ -7627,11 +7627,11 @@
 Scenario 2 - Description-only edit flags nothing
 Given an Event has confirmed venue and equipment arrangements When only its Event description is edited Then no arrangements are flagged
 Scenario 3 - Affected Session arrangements shown first
-Given a change affects confirmed arrangements When I save it Then I am shown the affected Session bookings, equipment reservations and staffed Technical Support requests before the change takes effect (T-103)
+Given a change affects confirmed arrangements When I save it Then I am shown the affected Session bookings, equipment reservations and staffed Technical Support requests before the change takes effect (T-104)
 Scenario 4 - Over-subscription warns only
 Given a change would make a Session or combined Event registration capacity lower than approved registrations When the change is saved Then I am warned and shown the over-subscription, and no Attendee is automatically removed or waitlisted
 Scenario 5 - Session date/time change flags its arrangements
-Given a Session date or time changes When the change takes effect Then that Session's venue booking and equipment reservations, and any staffed Technical Support request overlapping its previous time, are flagged for reconfirmation; an Event-wide date/time change flags all of its Session arrangements and every staffed Technical Support request; a flagged Technical Support request counts as outstanding for readiness until Technical Support Staff reconfirm it at the new time (T-103)
+Given a Session date or time changes When the change takes effect Then that Session's venue booking and equipment reservations, and any staffed Technical Support request overlapping its previous time, are flagged for reconfirmation; an Event-wide date/time change flags all of its Session arrangements and every staffed Technical Support request; a flagged Technical Support request counts as outstanding for readiness until Technical Support Staff reconfirm it at the new time (T-104)
 Scenario 6 - Affected staff notified
 Given a change flags a venue, equipment or Technical Support staffing arrangement When the affected arrangements are identified Then the assigned Venue Staff and Technical Support Staff are notified
 Checklist
@@ -7640,7 +7640,7 @@
 - Show affected Session bookings/reservations before applying a change
 - Warn about over-subscription without automatically removing or waitlisting Attendees
 - Flag the affected Session or all Sessions for date/time changes as appropriate
-- Flag staffed Technical Support requests on a date/time change and let Technical Support Staff reconfirm them at the new time (T-103)
+- Flag staffed Technical Support requests on a date/time change and let Technical Support Staff reconfirm them at the new time (T-104)
 - Notify staff responsible for the affected arrangements</t>
         </is>
       </c>
@@ -7649,7 +7649,7 @@
       </c>
       <c r="H69" s="2" t="inlineStr">
         <is>
-          <t>C-05, T-16, B-05, B-11, C-67, T-68, O-27, C-107, T-79, T-103</t>
+          <t>C-05, T-16, B-05, B-11, C-67, T-68, O-27, C-107, T-79, T-104</t>
         </is>
       </c>
       <c r="I69" s="2" t="inlineStr"/>

</xml_diff>